<commit_message>
Update Excel template with user's version
</commit_message>
<xml_diff>
--- a/server/export-template.xlsx
+++ b/server/export-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DD1AA6-34D4-41F2-90BF-3414268F2818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C5002F-6D32-4D1F-8C4E-12BA2845B87F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="771" xr2:uid="{184F55A4-A313-4B03-92E4-92DF68C567C7}"/>
   </bookViews>
@@ -13,19 +13,20 @@
     <sheet name="Project Tasks" sheetId="3" r:id="rId3"/>
     <sheet name="Projects" sheetId="4" r:id="rId4"/>
     <sheet name="Responsibilities" sheetId="5" r:id="rId5"/>
-    <sheet name="People" sheetId="6" r:id="rId6"/>
-    <sheet name="Places" sheetId="7" r:id="rId7"/>
-    <sheet name="Things" sheetId="8" r:id="rId8"/>
-    <sheet name="Providers" sheetId="9" r:id="rId9"/>
-    <sheet name="Conditions" sheetId="10" r:id="rId10"/>
-    <sheet name="Task Completions" sheetId="11" r:id="rId11"/>
+    <sheet name="Roles" sheetId="12" r:id="rId6"/>
+    <sheet name="People" sheetId="6" r:id="rId7"/>
+    <sheet name="Places" sheetId="7" r:id="rId8"/>
+    <sheet name="Things" sheetId="8" r:id="rId9"/>
+    <sheet name="Providers" sheetId="9" r:id="rId10"/>
+    <sheet name="Conditions" sheetId="10" r:id="rId11"/>
+    <sheet name="Task Completions" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="309">
   <si>
     <t>Export Date</t>
   </si>
@@ -1655,6 +1656,99 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>236</v>
+      </c>
+      <c r="D4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1761,7 +1855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4432,6 +4526,85 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91BF75C3-83C1-4543-898D-98483469DB31}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4552,7 +4725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4743,7 +4916,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4932,97 +5105,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>306</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>301</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>301</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>302</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>302</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>302</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>236</v>
-      </c>
-      <c r="D4" t="s">
-        <v>195</v>
-      </c>
-      <c r="F4" t="s">
-        <v>237</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
 </file>
</xml_diff>